<commit_message>
docs(qa): pruebas de API del Sprint 4 (asistencia diaria y esquema de medicación) en el ciclo de pruebas
</commit_message>
<xml_diff>
--- a/docs/qa/Ciclos_de_prueba_Sprint_1-4.xlsx
+++ b/docs/qa/Ciclos_de_prueba_Sprint_1-4.xlsx
@@ -12,6 +12,7 @@
     <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Ciclo - Sprint 3" sheetId="3" state="visible" r:id="rId3"/>
     <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Ciclo - Sprint 4" sheetId="4" state="visible" r:id="rId4"/>
     <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Ciclo - Seguridad y carga" sheetId="5" state="visible" r:id="rId5"/>
+    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Ciclo - Sprint 4 (API)" sheetId="6" state="visible" r:id="rId6"/>
   </sheets>
   <definedNames/>
   <calcPr calcId="124519" fullCalcOnLoad="1"/>
@@ -11133,4 +11134,1117 @@
   </dataValidations>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
 </worksheet>
+</file>
+
+<file path=xl/worksheets/sheet6.xml><?xml version="1.0" encoding="utf-8"?>
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
+  <sheetPr>
+    <outlinePr summaryBelow="1" summaryRight="1"/>
+    <pageSetUpPr/>
+  </sheetPr>
+  <dimension ref="A1:K24"/>
+  <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
+  <cols>
+    <col width="12" customWidth="1" min="1" max="1"/>
+    <col width="22" customWidth="1" min="2" max="2"/>
+    <col width="30" customWidth="1" min="3" max="3"/>
+    <col width="35" customWidth="1" min="4" max="4"/>
+    <col width="35" customWidth="1" min="5" max="5"/>
+    <col width="35" customWidth="1" min="6" max="6"/>
+    <col width="18" customWidth="1" min="7" max="7"/>
+    <col width="20" customWidth="1" min="8" max="8"/>
+    <col width="18" customWidth="1" min="9" max="9"/>
+    <col width="14" customWidth="1" min="10" max="10"/>
+    <col width="25" customWidth="1" min="11" max="11"/>
+  </cols>
+  <sheetData>
+    <row r="1" ht="40" customHeight="1">
+      <c r="A1" s="1" t="inlineStr">
+        <is>
+          <t>PLANILLA DE EJECUCIÓN DE CICLO DE PRUEBAS — Sprint 4 — endpoints ya desarrollados (asistencia diaria SCRUM-216 y esquema de medicación SCRUM-232), API local, 17/10/2026</t>
+        </is>
+      </c>
+    </row>
+    <row r="2" ht="15" customHeight="1"/>
+    <row r="3" ht="28" customHeight="1">
+      <c r="A3" s="2" t="inlineStr">
+        <is>
+          <t>ID Caso</t>
+        </is>
+      </c>
+      <c r="B3" s="2" t="inlineStr">
+        <is>
+          <t>Módulo / Componente</t>
+        </is>
+      </c>
+      <c r="C3" s="2" t="inlineStr">
+        <is>
+          <t>Título del Caso de Prueba</t>
+        </is>
+      </c>
+      <c r="D3" s="2" t="inlineStr">
+        <is>
+          <t>Pasos de Ejecución</t>
+        </is>
+      </c>
+      <c r="E3" s="2" t="inlineStr">
+        <is>
+          <t>Resultado Esperado</t>
+        </is>
+      </c>
+      <c r="F3" s="2" t="inlineStr">
+        <is>
+          <t>Resultado Real</t>
+        </is>
+      </c>
+      <c r="G3" s="2" t="inlineStr">
+        <is>
+          <t>Estado</t>
+        </is>
+      </c>
+      <c r="H3" s="2" t="inlineStr">
+        <is>
+          <t>ID Bug (Jira/Tool)</t>
+        </is>
+      </c>
+      <c r="I3" s="2" t="inlineStr">
+        <is>
+          <t>Ejecutado Por</t>
+        </is>
+      </c>
+      <c r="J3" s="2" t="inlineStr">
+        <is>
+          <t>Fecha</t>
+        </is>
+      </c>
+      <c r="K3" s="2" t="inlineStr">
+        <is>
+          <t>Comentarios</t>
+        </is>
+      </c>
+    </row>
+    <row r="4" ht="22" customHeight="1">
+      <c r="A4" s="3" t="inlineStr">
+        <is>
+          <t>S4-A01</t>
+        </is>
+      </c>
+      <c r="B4" s="4" t="inlineStr">
+        <is>
+          <t>Asistencia diaria (SCRUM-54 / 216)</t>
+        </is>
+      </c>
+      <c r="C4" s="4" t="inlineStr">
+        <is>
+          <t>Referente registra la asistencia de una persona en Hogar de día (204)</t>
+        </is>
+      </c>
+      <c r="D4" s="4" t="inlineStr">
+        <is>
+          <t>1. Iniciar sesión con el rol indicado en el título (Referente por defecto)
+2. POST /api/attendances con el dato del caso</t>
+        </is>
+      </c>
+      <c r="E4" s="4" t="inlineStr">
+        <is>
+          <t>Referente registra la asistencia de una persona en Hogar de día (204)</t>
+        </is>
+      </c>
+      <c r="F4" s="4" t="inlineStr">
+        <is>
+          <t>Respuesta de la API: status=204</t>
+        </is>
+      </c>
+      <c r="G4" s="5" t="inlineStr">
+        <is>
+          <t>PASÓ</t>
+        </is>
+      </c>
+      <c r="H4" s="3" t="n"/>
+      <c r="I4" s="3" t="inlineStr">
+        <is>
+          <t>QA (script sprint4-api-flows.mjs)</t>
+        </is>
+      </c>
+      <c r="J4" s="7" t="n">
+        <v>46312</v>
+      </c>
+      <c r="K4" s="4" t="inlineStr">
+        <is>
+          <t>Observación: la actividad viaja como número (0 = Hogar de día, 1 = Casa de Convivencia) y no como texto; el front debe enviarla así.</t>
+        </is>
+      </c>
+    </row>
+    <row r="5" ht="22" customHeight="1">
+      <c r="A5" s="3" t="inlineStr">
+        <is>
+          <t>S4-A02</t>
+        </is>
+      </c>
+      <c r="B5" s="4" t="inlineStr">
+        <is>
+          <t>Asistencia diaria (SCRUM-54 / 216)</t>
+        </is>
+      </c>
+      <c r="C5" s="4" t="inlineStr">
+        <is>
+          <t>La misma persona, actividad y fecha no se registra dos veces (409)</t>
+        </is>
+      </c>
+      <c r="D5" s="4" t="inlineStr">
+        <is>
+          <t>1. Iniciar sesión con el rol indicado en el título (Referente por defecto)
+2. POST /api/attendances con el dato del caso</t>
+        </is>
+      </c>
+      <c r="E5" s="4" t="inlineStr">
+        <is>
+          <t>La misma persona, actividad y fecha no se registra dos veces (409)</t>
+        </is>
+      </c>
+      <c r="F5" s="4" t="inlineStr">
+        <is>
+          <t>Respuesta de la API: status=409 Ya existe un registro de asistencia para esa persona, actividad y fecha.</t>
+        </is>
+      </c>
+      <c r="G5" s="5" t="inlineStr">
+        <is>
+          <t>PASÓ</t>
+        </is>
+      </c>
+      <c r="H5" s="3" t="n"/>
+      <c r="I5" s="3" t="inlineStr">
+        <is>
+          <t>QA (script sprint4-api-flows.mjs)</t>
+        </is>
+      </c>
+      <c r="J5" s="7" t="n">
+        <v>46312</v>
+      </c>
+      <c r="K5" s="4" t="n"/>
+    </row>
+    <row r="6" ht="22" customHeight="1">
+      <c r="A6" s="3" t="inlineStr">
+        <is>
+          <t>S4-A03</t>
+        </is>
+      </c>
+      <c r="B6" s="4" t="inlineStr">
+        <is>
+          <t>Asistencia diaria (SCRUM-54 / 216)</t>
+        </is>
+      </c>
+      <c r="C6" s="4" t="inlineStr">
+        <is>
+          <t>La misma persona sí puede asistir a otra actividad el mismo día (204)</t>
+        </is>
+      </c>
+      <c r="D6" s="4" t="inlineStr">
+        <is>
+          <t>1. Iniciar sesión con el rol indicado en el título (Referente por defecto)
+2. POST /api/attendances con el dato del caso</t>
+        </is>
+      </c>
+      <c r="E6" s="4" t="inlineStr">
+        <is>
+          <t>La misma persona sí puede asistir a otra actividad el mismo día (204)</t>
+        </is>
+      </c>
+      <c r="F6" s="4" t="inlineStr">
+        <is>
+          <t>Respuesta de la API: status=204</t>
+        </is>
+      </c>
+      <c r="G6" s="5" t="inlineStr">
+        <is>
+          <t>PASÓ</t>
+        </is>
+      </c>
+      <c r="H6" s="3" t="n"/>
+      <c r="I6" s="3" t="inlineStr">
+        <is>
+          <t>QA (script sprint4-api-flows.mjs)</t>
+        </is>
+      </c>
+      <c r="J6" s="7" t="n">
+        <v>46312</v>
+      </c>
+      <c r="K6" s="4" t="n"/>
+    </row>
+    <row r="7" ht="22" customHeight="1">
+      <c r="A7" s="3" t="inlineStr">
+        <is>
+          <t>S4-A04</t>
+        </is>
+      </c>
+      <c r="B7" s="4" t="inlineStr">
+        <is>
+          <t>Asistencia diaria (SCRUM-54 / 216)</t>
+        </is>
+      </c>
+      <c r="C7" s="4" t="inlineStr">
+        <is>
+          <t>Se acepta un conteo de personas sin ficha (204)</t>
+        </is>
+      </c>
+      <c r="D7" s="4" t="inlineStr">
+        <is>
+          <t>1. Iniciar sesión con el rol indicado en el título (Referente por defecto)
+2. POST /api/attendances con el dato del caso</t>
+        </is>
+      </c>
+      <c r="E7" s="4" t="inlineStr">
+        <is>
+          <t>Se acepta un conteo de personas sin ficha (204)</t>
+        </is>
+      </c>
+      <c r="F7" s="4" t="inlineStr">
+        <is>
+          <t>Respuesta de la API: status=204</t>
+        </is>
+      </c>
+      <c r="G7" s="5" t="inlineStr">
+        <is>
+          <t>PASÓ</t>
+        </is>
+      </c>
+      <c r="H7" s="3" t="n"/>
+      <c r="I7" s="3" t="inlineStr">
+        <is>
+          <t>QA (script sprint4-api-flows.mjs)</t>
+        </is>
+      </c>
+      <c r="J7" s="7" t="n">
+        <v>46312</v>
+      </c>
+      <c r="K7" s="4" t="n"/>
+    </row>
+    <row r="8" ht="22" customHeight="1">
+      <c r="A8" s="3" t="inlineStr">
+        <is>
+          <t>S4-A05</t>
+        </is>
+      </c>
+      <c r="B8" s="4" t="inlineStr">
+        <is>
+          <t>Asistencia diaria (SCRUM-54 / 216)</t>
+        </is>
+      </c>
+      <c r="C8" s="4" t="inlineStr">
+        <is>
+          <t>Un conteo negativo se rechaza con mensaje de validación (400)</t>
+        </is>
+      </c>
+      <c r="D8" s="4" t="inlineStr">
+        <is>
+          <t>1. Iniciar sesión con el rol indicado en el título (Referente por defecto)
+2. POST /api/attendances con el dato del caso</t>
+        </is>
+      </c>
+      <c r="E8" s="4" t="inlineStr">
+        <is>
+          <t>Un conteo negativo se rechaza con mensaje de validación (400)</t>
+        </is>
+      </c>
+      <c r="F8" s="4" t="inlineStr">
+        <is>
+          <t>Respuesta de la API: status=400</t>
+        </is>
+      </c>
+      <c r="G8" s="5" t="inlineStr">
+        <is>
+          <t>PASÓ</t>
+        </is>
+      </c>
+      <c r="H8" s="3" t="n"/>
+      <c r="I8" s="3" t="inlineStr">
+        <is>
+          <t>QA (script sprint4-api-flows.mjs)</t>
+        </is>
+      </c>
+      <c r="J8" s="7" t="n">
+        <v>46312</v>
+      </c>
+      <c r="K8" s="4" t="n"/>
+    </row>
+    <row r="9" ht="22" customHeight="1">
+      <c r="A9" s="3" t="inlineStr">
+        <is>
+          <t>S4-A06</t>
+        </is>
+      </c>
+      <c r="B9" s="4" t="inlineStr">
+        <is>
+          <t>Asistencia diaria (SCRUM-54 / 216)</t>
+        </is>
+      </c>
+      <c r="C9" s="4" t="inlineStr">
+        <is>
+          <t>No se registra asistencia con fecha futura (400)</t>
+        </is>
+      </c>
+      <c r="D9" s="4" t="inlineStr">
+        <is>
+          <t>1. Iniciar sesión con el rol indicado en el título (Referente por defecto)
+2. POST /api/attendances con el dato del caso</t>
+        </is>
+      </c>
+      <c r="E9" s="4" t="inlineStr">
+        <is>
+          <t>No se registra asistencia con fecha futura (400)</t>
+        </is>
+      </c>
+      <c r="F9" s="4" t="inlineStr">
+        <is>
+          <t>Respuesta de la API: status=400</t>
+        </is>
+      </c>
+      <c r="G9" s="5" t="inlineStr">
+        <is>
+          <t>PASÓ</t>
+        </is>
+      </c>
+      <c r="H9" s="3" t="n"/>
+      <c r="I9" s="3" t="inlineStr">
+        <is>
+          <t>QA (script sprint4-api-flows.mjs)</t>
+        </is>
+      </c>
+      <c r="J9" s="7" t="n">
+        <v>46312</v>
+      </c>
+      <c r="K9" s="4" t="n"/>
+    </row>
+    <row r="10" ht="22" customHeight="1">
+      <c r="A10" s="3" t="inlineStr">
+        <is>
+          <t>S4-A07</t>
+        </is>
+      </c>
+      <c r="B10" s="4" t="inlineStr">
+        <is>
+          <t>Asistencia diaria (SCRUM-54 / 216)</t>
+        </is>
+      </c>
+      <c r="C10" s="4" t="inlineStr">
+        <is>
+          <t>Una persona inexistente responde 404</t>
+        </is>
+      </c>
+      <c r="D10" s="4" t="inlineStr">
+        <is>
+          <t>1. Iniciar sesión con el rol indicado en el título (Referente por defecto)
+2. POST /api/attendances con el dato del caso</t>
+        </is>
+      </c>
+      <c r="E10" s="4" t="inlineStr">
+        <is>
+          <t>Una persona inexistente responde 404</t>
+        </is>
+      </c>
+      <c r="F10" s="4" t="inlineStr">
+        <is>
+          <t>Respuesta de la API: status=404</t>
+        </is>
+      </c>
+      <c r="G10" s="5" t="inlineStr">
+        <is>
+          <t>PASÓ</t>
+        </is>
+      </c>
+      <c r="H10" s="3" t="n"/>
+      <c r="I10" s="3" t="inlineStr">
+        <is>
+          <t>QA (script sprint4-api-flows.mjs)</t>
+        </is>
+      </c>
+      <c r="J10" s="7" t="n">
+        <v>46312</v>
+      </c>
+      <c r="K10" s="4" t="n"/>
+    </row>
+    <row r="11" ht="22" customHeight="1">
+      <c r="A11" s="3" t="inlineStr">
+        <is>
+          <t>S4-A08</t>
+        </is>
+      </c>
+      <c r="B11" s="4" t="inlineStr">
+        <is>
+          <t>Asistencia diaria (SCRUM-54 / 216)</t>
+        </is>
+      </c>
+      <c r="C11" s="4" t="inlineStr">
+        <is>
+          <t>Una actividad inválida se rechaza sin error 500 (400)</t>
+        </is>
+      </c>
+      <c r="D11" s="4" t="inlineStr">
+        <is>
+          <t>1. Iniciar sesión con el rol indicado en el título (Referente por defecto)
+2. POST /api/attendances con el dato del caso</t>
+        </is>
+      </c>
+      <c r="E11" s="4" t="inlineStr">
+        <is>
+          <t>Una actividad inválida se rechaza sin error 500 (400)</t>
+        </is>
+      </c>
+      <c r="F11" s="4" t="inlineStr">
+        <is>
+          <t>Respuesta de la API: status=400</t>
+        </is>
+      </c>
+      <c r="G11" s="5" t="inlineStr">
+        <is>
+          <t>PASÓ</t>
+        </is>
+      </c>
+      <c r="H11" s="3" t="n"/>
+      <c r="I11" s="3" t="inlineStr">
+        <is>
+          <t>QA (script sprint4-api-flows.mjs)</t>
+        </is>
+      </c>
+      <c r="J11" s="7" t="n">
+        <v>46312</v>
+      </c>
+      <c r="K11" s="4" t="n"/>
+    </row>
+    <row r="12" ht="22" customHeight="1">
+      <c r="A12" s="3" t="inlineStr">
+        <is>
+          <t>S4-A09</t>
+        </is>
+      </c>
+      <c r="B12" s="4" t="inlineStr">
+        <is>
+          <t>Asistencia diaria (SCRUM-54 / 216)</t>
+        </is>
+      </c>
+      <c r="C12" s="4" t="inlineStr">
+        <is>
+          <t>Sin sesión responde 401</t>
+        </is>
+      </c>
+      <c r="D12" s="4" t="inlineStr">
+        <is>
+          <t>1. Iniciar sesión con el rol indicado en el título (Referente por defecto)
+2. POST /api/attendances con el dato del caso</t>
+        </is>
+      </c>
+      <c r="E12" s="4" t="inlineStr">
+        <is>
+          <t>Sin sesión responde 401</t>
+        </is>
+      </c>
+      <c r="F12" s="4" t="inlineStr">
+        <is>
+          <t>Respuesta de la API: status=401</t>
+        </is>
+      </c>
+      <c r="G12" s="5" t="inlineStr">
+        <is>
+          <t>PASÓ</t>
+        </is>
+      </c>
+      <c r="H12" s="3" t="n"/>
+      <c r="I12" s="3" t="inlineStr">
+        <is>
+          <t>QA (script sprint4-api-flows.mjs)</t>
+        </is>
+      </c>
+      <c r="J12" s="7" t="n">
+        <v>46312</v>
+      </c>
+      <c r="K12" s="4" t="n"/>
+    </row>
+    <row r="13" ht="22" customHeight="1">
+      <c r="A13" s="3" t="inlineStr">
+        <is>
+          <t>S4-A10</t>
+        </is>
+      </c>
+      <c r="B13" s="4" t="inlineStr">
+        <is>
+          <t>Asistencia diaria (SCRUM-54 / 216)</t>
+        </is>
+      </c>
+      <c r="C13" s="4" t="inlineStr">
+        <is>
+          <t>Escucha puede registrar asistencia del día a día del Centro Barrial (204)</t>
+        </is>
+      </c>
+      <c r="D13" s="4" t="inlineStr">
+        <is>
+          <t>1. Iniciar sesión con el rol indicado en el título (Referente por defecto)
+2. POST /api/attendances con el dato del caso</t>
+        </is>
+      </c>
+      <c r="E13" s="4" t="inlineStr">
+        <is>
+          <t>Escucha puede registrar asistencia del día a día del Centro Barrial (204)</t>
+        </is>
+      </c>
+      <c r="F13" s="4" t="inlineStr">
+        <is>
+          <t>Respuesta de la API: status=204</t>
+        </is>
+      </c>
+      <c r="G13" s="5" t="inlineStr">
+        <is>
+          <t>PASÓ</t>
+        </is>
+      </c>
+      <c r="H13" s="3" t="n"/>
+      <c r="I13" s="3" t="inlineStr">
+        <is>
+          <t>QA (script sprint4-api-flows.mjs)</t>
+        </is>
+      </c>
+      <c r="J13" s="7" t="n">
+        <v>46312</v>
+      </c>
+      <c r="K13" s="4" t="n"/>
+    </row>
+    <row r="14" ht="22" customHeight="1">
+      <c r="A14" s="3" t="inlineStr">
+        <is>
+          <t>S4-A11</t>
+        </is>
+      </c>
+      <c r="B14" s="4" t="inlineStr">
+        <is>
+          <t>Asistencia diaria (SCRUM-54 / 216)</t>
+        </is>
+      </c>
+      <c r="C14" s="4" t="inlineStr">
+        <is>
+          <t>Coordinador de Casona registra asistencia de un residente (204)</t>
+        </is>
+      </c>
+      <c r="D14" s="4" t="inlineStr">
+        <is>
+          <t>1. Iniciar sesión con el rol indicado en el título (Referente por defecto)
+2. POST /api/attendances con el dato del caso</t>
+        </is>
+      </c>
+      <c r="E14" s="4" t="inlineStr">
+        <is>
+          <t>Coordinador de Casona registra asistencia de un residente (204)</t>
+        </is>
+      </c>
+      <c r="F14" s="4" t="inlineStr">
+        <is>
+          <t>Respuesta de la API: status=204</t>
+        </is>
+      </c>
+      <c r="G14" s="5" t="inlineStr">
+        <is>
+          <t>PASÓ</t>
+        </is>
+      </c>
+      <c r="H14" s="3" t="n"/>
+      <c r="I14" s="3" t="inlineStr">
+        <is>
+          <t>QA (script sprint4-api-flows.mjs)</t>
+        </is>
+      </c>
+      <c r="J14" s="7" t="n">
+        <v>46312</v>
+      </c>
+      <c r="K14" s="4" t="n"/>
+    </row>
+    <row r="15" ht="22" customHeight="1">
+      <c r="A15" s="3" t="inlineStr">
+        <is>
+          <t>S4-M01</t>
+        </is>
+      </c>
+      <c r="B15" s="4" t="inlineStr">
+        <is>
+          <t>Esquema de medicación (SCRUM-59 / 232)</t>
+        </is>
+      </c>
+      <c r="C15" s="4" t="inlineStr">
+        <is>
+          <t>Referente carga un esquema a un Residente con evaluación vigente (201 con el esquema completo)</t>
+        </is>
+      </c>
+      <c r="D15" s="4" t="inlineStr">
+        <is>
+          <t>1. Iniciar sesión con el rol indicado en el título (Referente por defecto)
+2. POST /api/persons/{id}/medication-schemes con el dato del caso</t>
+        </is>
+      </c>
+      <c r="E15" s="4" t="inlineStr">
+        <is>
+          <t>Referente carga un esquema a un Residente con evaluación vigente (201 con el esquema completo)</t>
+        </is>
+      </c>
+      <c r="F15" s="4" t="inlineStr">
+        <is>
+          <t>Respuesta de la API: status=201 Medicamento de prueba A pendingStock=false</t>
+        </is>
+      </c>
+      <c r="G15" s="5" t="inlineStr">
+        <is>
+          <t>PASÓ</t>
+        </is>
+      </c>
+      <c r="H15" s="3" t="n"/>
+      <c r="I15" s="3" t="inlineStr">
+        <is>
+          <t>QA (script sprint4-api-flows.mjs)</t>
+        </is>
+      </c>
+      <c r="J15" s="7" t="n">
+        <v>46312</v>
+      </c>
+      <c r="K15" s="4" t="n"/>
+    </row>
+    <row r="16" ht="22" customHeight="1">
+      <c r="A16" s="3" t="inlineStr">
+        <is>
+          <t>S4-M02</t>
+        </is>
+      </c>
+      <c r="B16" s="4" t="inlineStr">
+        <is>
+          <t>Esquema de medicación (SCRUM-59 / 232)</t>
+        </is>
+      </c>
+      <c r="C16" s="4" t="inlineStr">
+        <is>
+          <t>Un esquema duplicado vigente se rechaza (409)</t>
+        </is>
+      </c>
+      <c r="D16" s="4" t="inlineStr">
+        <is>
+          <t>1. Iniciar sesión con el rol indicado en el título (Referente por defecto)
+2. POST /api/persons/{id}/medication-schemes con el dato del caso</t>
+        </is>
+      </c>
+      <c r="E16" s="4" t="inlineStr">
+        <is>
+          <t>Un esquema duplicado vigente se rechaza (409)</t>
+        </is>
+      </c>
+      <c r="F16" s="4" t="inlineStr">
+        <is>
+          <t>Respuesta de la API: status=409 Ya existe un esquema vigente con ese medicamento y horario para la persona.</t>
+        </is>
+      </c>
+      <c r="G16" s="5" t="inlineStr">
+        <is>
+          <t>PASÓ</t>
+        </is>
+      </c>
+      <c r="H16" s="3" t="n"/>
+      <c r="I16" s="3" t="inlineStr">
+        <is>
+          <t>QA (script sprint4-api-flows.mjs)</t>
+        </is>
+      </c>
+      <c r="J16" s="7" t="n">
+        <v>46312</v>
+      </c>
+      <c r="K16" s="4" t="n"/>
+    </row>
+    <row r="17" ht="22" customHeight="1">
+      <c r="A17" s="3" t="inlineStr">
+        <is>
+          <t>S4-M03</t>
+        </is>
+      </c>
+      <c r="B17" s="4" t="inlineStr">
+        <is>
+          <t>Esquema de medicación (SCRUM-59 / 232)</t>
+        </is>
+      </c>
+      <c r="C17" s="4" t="inlineStr">
+        <is>
+          <t>Un medicamento sin stock se carga igual y queda marcado como pendiente de stock (201)</t>
+        </is>
+      </c>
+      <c r="D17" s="4" t="inlineStr">
+        <is>
+          <t>1. Iniciar sesión con el rol indicado en el título (Referente por defecto)
+2. POST /api/persons/{id}/medication-schemes con el dato del caso</t>
+        </is>
+      </c>
+      <c r="E17" s="4" t="inlineStr">
+        <is>
+          <t>Un medicamento sin stock se carga igual y queda marcado como pendiente de stock (201)</t>
+        </is>
+      </c>
+      <c r="F17" s="4" t="inlineStr">
+        <is>
+          <t>Respuesta de la API: status=201 pendingStock=true</t>
+        </is>
+      </c>
+      <c r="G17" s="5" t="inlineStr">
+        <is>
+          <t>PASÓ</t>
+        </is>
+      </c>
+      <c r="H17" s="3" t="n"/>
+      <c r="I17" s="3" t="inlineStr">
+        <is>
+          <t>QA (script sprint4-api-flows.mjs)</t>
+        </is>
+      </c>
+      <c r="J17" s="7" t="n">
+        <v>46312</v>
+      </c>
+      <c r="K17" s="4" t="n"/>
+    </row>
+    <row r="18" ht="22" customHeight="1">
+      <c r="A18" s="3" t="inlineStr">
+        <is>
+          <t>S4-M04</t>
+        </is>
+      </c>
+      <c r="B18" s="4" t="inlineStr">
+        <is>
+          <t>Esquema de medicación (SCRUM-59 / 232)</t>
+        </is>
+      </c>
+      <c r="C18" s="4" t="inlineStr">
+        <is>
+          <t>Sin evaluación psiquiátrica vigente no se puede cargar el esquema (4xx)</t>
+        </is>
+      </c>
+      <c r="D18" s="4" t="inlineStr">
+        <is>
+          <t>1. Iniciar sesión con el rol indicado en el título (Referente por defecto)
+2. POST /api/persons/{id}/medication-schemes con el dato del caso</t>
+        </is>
+      </c>
+      <c r="E18" s="4" t="inlineStr">
+        <is>
+          <t>Sin evaluación psiquiátrica vigente no se puede cargar el esquema (4xx)</t>
+        </is>
+      </c>
+      <c r="F18" s="4" t="inlineStr">
+        <is>
+          <t>Respuesta de la API: status=400 No se puede cargar medicación: la persona no tiene una evaluación psiquiátrica vigente.</t>
+        </is>
+      </c>
+      <c r="G18" s="5" t="inlineStr">
+        <is>
+          <t>PASÓ</t>
+        </is>
+      </c>
+      <c r="H18" s="3" t="n"/>
+      <c r="I18" s="3" t="inlineStr">
+        <is>
+          <t>QA (script sprint4-api-flows.mjs)</t>
+        </is>
+      </c>
+      <c r="J18" s="7" t="n">
+        <v>46312</v>
+      </c>
+      <c r="K18" s="4" t="n"/>
+    </row>
+    <row r="19" ht="22" customHeight="1">
+      <c r="A19" s="3" t="inlineStr">
+        <is>
+          <t>S4-M05</t>
+        </is>
+      </c>
+      <c r="B19" s="4" t="inlineStr">
+        <is>
+          <t>Esquema de medicación (SCRUM-59 / 232)</t>
+        </is>
+      </c>
+      <c r="C19" s="4" t="inlineStr">
+        <is>
+          <t>Escucha no puede cargar esquemas (403)</t>
+        </is>
+      </c>
+      <c r="D19" s="4" t="inlineStr">
+        <is>
+          <t>1. Iniciar sesión con el rol indicado en el título (Referente por defecto)
+2. POST /api/persons/{id}/medication-schemes con el dato del caso</t>
+        </is>
+      </c>
+      <c r="E19" s="4" t="inlineStr">
+        <is>
+          <t>Escucha no puede cargar esquemas (403)</t>
+        </is>
+      </c>
+      <c r="F19" s="4" t="inlineStr">
+        <is>
+          <t>Respuesta de la API: status=403</t>
+        </is>
+      </c>
+      <c r="G19" s="5" t="inlineStr">
+        <is>
+          <t>PASÓ</t>
+        </is>
+      </c>
+      <c r="H19" s="3" t="n"/>
+      <c r="I19" s="3" t="inlineStr">
+        <is>
+          <t>QA (script sprint4-api-flows.mjs)</t>
+        </is>
+      </c>
+      <c r="J19" s="7" t="n">
+        <v>46312</v>
+      </c>
+      <c r="K19" s="4" t="n"/>
+    </row>
+    <row r="20" ht="22" customHeight="1">
+      <c r="A20" s="3" t="inlineStr">
+        <is>
+          <t>S4-M06</t>
+        </is>
+      </c>
+      <c r="B20" s="4" t="inlineStr">
+        <is>
+          <t>Esquema de medicación (SCRUM-59 / 232)</t>
+        </is>
+      </c>
+      <c r="C20" s="4" t="inlineStr">
+        <is>
+          <t>Una hora inválida se rechaza (400)</t>
+        </is>
+      </c>
+      <c r="D20" s="4" t="inlineStr">
+        <is>
+          <t>1. Iniciar sesión con el rol indicado en el título (Referente por defecto)
+2. POST /api/persons/{id}/medication-schemes con el dato del caso</t>
+        </is>
+      </c>
+      <c r="E20" s="4" t="inlineStr">
+        <is>
+          <t>Una hora inválida se rechaza (400)</t>
+        </is>
+      </c>
+      <c r="F20" s="4" t="inlineStr">
+        <is>
+          <t>Respuesta de la API: status=400</t>
+        </is>
+      </c>
+      <c r="G20" s="5" t="inlineStr">
+        <is>
+          <t>PASÓ</t>
+        </is>
+      </c>
+      <c r="H20" s="3" t="n"/>
+      <c r="I20" s="3" t="inlineStr">
+        <is>
+          <t>QA (script sprint4-api-flows.mjs)</t>
+        </is>
+      </c>
+      <c r="J20" s="7" t="n">
+        <v>46312</v>
+      </c>
+      <c r="K20" s="4" t="n"/>
+    </row>
+    <row r="21" ht="22" customHeight="1">
+      <c r="A21" s="3" t="inlineStr">
+        <is>
+          <t>S4-M07</t>
+        </is>
+      </c>
+      <c r="B21" s="4" t="inlineStr">
+        <is>
+          <t>Esquema de medicación (SCRUM-59 / 232)</t>
+        </is>
+      </c>
+      <c r="C21" s="4" t="inlineStr">
+        <is>
+          <t>La dosis vacía se rechaza (400)</t>
+        </is>
+      </c>
+      <c r="D21" s="4" t="inlineStr">
+        <is>
+          <t>1. Iniciar sesión con el rol indicado en el título (Referente por defecto)
+2. POST /api/persons/{id}/medication-schemes con el dato del caso</t>
+        </is>
+      </c>
+      <c r="E21" s="4" t="inlineStr">
+        <is>
+          <t>La dosis vacía se rechaza (400)</t>
+        </is>
+      </c>
+      <c r="F21" s="4" t="inlineStr">
+        <is>
+          <t>Respuesta de la API: status=400</t>
+        </is>
+      </c>
+      <c r="G21" s="5" t="inlineStr">
+        <is>
+          <t>PASÓ</t>
+        </is>
+      </c>
+      <c r="H21" s="3" t="n"/>
+      <c r="I21" s="3" t="inlineStr">
+        <is>
+          <t>QA (script sprint4-api-flows.mjs)</t>
+        </is>
+      </c>
+      <c r="J21" s="7" t="n">
+        <v>46312</v>
+      </c>
+      <c r="K21" s="4" t="n"/>
+    </row>
+    <row r="22" ht="22" customHeight="1">
+      <c r="A22" s="3" t="inlineStr">
+        <is>
+          <t>S4-M08</t>
+        </is>
+      </c>
+      <c r="B22" s="4" t="inlineStr">
+        <is>
+          <t>Esquema de medicación (SCRUM-59 / 232)</t>
+        </is>
+      </c>
+      <c r="C22" s="4" t="inlineStr">
+        <is>
+          <t>Un medicamento fuera del catálogo responde 404</t>
+        </is>
+      </c>
+      <c r="D22" s="4" t="inlineStr">
+        <is>
+          <t>1. Iniciar sesión con el rol indicado en el título (Referente por defecto)
+2. POST /api/persons/{id}/medication-schemes con el dato del caso</t>
+        </is>
+      </c>
+      <c r="E22" s="4" t="inlineStr">
+        <is>
+          <t>Un medicamento fuera del catálogo responde 404</t>
+        </is>
+      </c>
+      <c r="F22" s="4" t="inlineStr">
+        <is>
+          <t>Respuesta de la API: status=404</t>
+        </is>
+      </c>
+      <c r="G22" s="5" t="inlineStr">
+        <is>
+          <t>PASÓ</t>
+        </is>
+      </c>
+      <c r="H22" s="3" t="n"/>
+      <c r="I22" s="3" t="inlineStr">
+        <is>
+          <t>QA (script sprint4-api-flows.mjs)</t>
+        </is>
+      </c>
+      <c r="J22" s="7" t="n">
+        <v>46312</v>
+      </c>
+      <c r="K22" s="4" t="n"/>
+    </row>
+    <row r="23" ht="22" customHeight="1">
+      <c r="A23" s="3" t="inlineStr">
+        <is>
+          <t>S4-M09</t>
+        </is>
+      </c>
+      <c r="B23" s="4" t="inlineStr">
+        <is>
+          <t>Esquema de medicación (SCRUM-59 / 232)</t>
+        </is>
+      </c>
+      <c r="C23" s="4" t="inlineStr">
+        <is>
+          <t>Una persona inexistente responde 404</t>
+        </is>
+      </c>
+      <c r="D23" s="4" t="inlineStr">
+        <is>
+          <t>1. Iniciar sesión con el rol indicado en el título (Referente por defecto)
+2. POST /api/persons/{id}/medication-schemes con el dato del caso</t>
+        </is>
+      </c>
+      <c r="E23" s="4" t="inlineStr">
+        <is>
+          <t>Una persona inexistente responde 404</t>
+        </is>
+      </c>
+      <c r="F23" s="4" t="inlineStr">
+        <is>
+          <t>Respuesta de la API: status=404</t>
+        </is>
+      </c>
+      <c r="G23" s="5" t="inlineStr">
+        <is>
+          <t>PASÓ</t>
+        </is>
+      </c>
+      <c r="H23" s="3" t="n"/>
+      <c r="I23" s="3" t="inlineStr">
+        <is>
+          <t>QA (script sprint4-api-flows.mjs)</t>
+        </is>
+      </c>
+      <c r="J23" s="7" t="n">
+        <v>46312</v>
+      </c>
+      <c r="K23" s="4" t="n"/>
+    </row>
+    <row r="24" ht="22" customHeight="1">
+      <c r="A24" s="3" t="inlineStr">
+        <is>
+          <t>S4-M10</t>
+        </is>
+      </c>
+      <c r="B24" s="4" t="inlineStr">
+        <is>
+          <t>Esquema de medicación (SCRUM-59 / 232)</t>
+        </is>
+      </c>
+      <c r="C24" s="4" t="inlineStr">
+        <is>
+          <t>Sin sesión responde 401</t>
+        </is>
+      </c>
+      <c r="D24" s="4" t="inlineStr">
+        <is>
+          <t>1. Iniciar sesión con el rol indicado en el título (Referente por defecto)
+2. POST /api/persons/{id}/medication-schemes con el dato del caso</t>
+        </is>
+      </c>
+      <c r="E24" s="4" t="inlineStr">
+        <is>
+          <t>Sin sesión responde 401</t>
+        </is>
+      </c>
+      <c r="F24" s="4" t="inlineStr">
+        <is>
+          <t>Respuesta de la API: status=401</t>
+        </is>
+      </c>
+      <c r="G24" s="5" t="inlineStr">
+        <is>
+          <t>PASÓ</t>
+        </is>
+      </c>
+      <c r="H24" s="3" t="n"/>
+      <c r="I24" s="3" t="inlineStr">
+        <is>
+          <t>QA (script sprint4-api-flows.mjs)</t>
+        </is>
+      </c>
+      <c r="J24" s="7" t="n">
+        <v>46312</v>
+      </c>
+      <c r="K24" s="4" t="n"/>
+    </row>
+    <row r="25" ht="22" customHeight="1"/>
+  </sheetData>
+  <mergeCells count="1">
+    <mergeCell ref="A1:K1"/>
+  </mergeCells>
+  <dataValidations count="1">
+    <dataValidation sqref="G4:G24" showDropDown="0" showInputMessage="0" showErrorMessage="0" allowBlank="0" type="list">
+      <formula1>"PASÓ,FALLÓ,BLOQUEADO,NO EJECUTADO"</formula1>
+    </dataValidation>
+  </dataValidations>
+  <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
+</worksheet>
 </file>
</xml_diff>